<commit_message>
generated products and stores and make sure its working perfectly
</commit_message>
<xml_diff>
--- a/generator/output/master/categories.xlsx
+++ b/generator/output/master/categories.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -465,21 +465,21 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>{'CAT001'}</t>
+          <t>CAT001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Maize Flour</t>
+          <t>Grocery</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Grocery</t>
+          <t>Food</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="E2" t="b">
         <v>0</v>
@@ -497,24 +497,24 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>{'CAT002'}</t>
+          <t>CAT002</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Rice</t>
+          <t>Dairy</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Grocery</t>
+          <t>Fresh Foods</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="E3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F3" s="1" t="n">
         <v>43831</v>
@@ -529,24 +529,24 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>{'CAT003'}</t>
+          <t>CAT003</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Sugar</t>
+          <t>Bakery</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Grocery</t>
+          <t>Fresh Foods</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="E4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F4" s="1" t="n">
         <v>43831</v>
@@ -561,24 +561,24 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>{'CAT004'}</t>
+          <t>CAT004</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Cooking Oil</t>
+          <t>Fresh Produce</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Grocery</t>
+          <t>Fresh Foods</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="E5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F5" s="1" t="n">
         <v>43831</v>
@@ -593,24 +593,24 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>{'CAT005'}</t>
+          <t>CAT005</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Salt</t>
+          <t>Meat &amp; Poultry</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Grocery</t>
+          <t>Fresh Foods</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="E6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F6" s="1" t="n">
         <v>43831</v>
@@ -625,12 +625,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>{'CAT006'}</t>
+          <t>CAT006</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Milk</t>
+          <t>Fish &amp; Seafood</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -639,7 +639,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="E7" t="b">
         <v>1</v>
@@ -657,17 +657,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>{'CAT007'}</t>
+          <t>CAT007</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Yoghurt</t>
+          <t>Frozen Foods</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Fresh Foods</t>
+          <t>Frozen</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -689,24 +689,24 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>{'CAT008'}</t>
+          <t>CAT008</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Cheese</t>
+          <t>Beverages</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Fresh Foods</t>
+          <t>Beverages</t>
         </is>
       </c>
       <c r="D9" t="n">
         <v>16</v>
       </c>
       <c r="E9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F9" s="1" t="n">
         <v>43831</v>
@@ -721,24 +721,24 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>{'CAT009'}</t>
+          <t>CAT009</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Butter</t>
+          <t>Juices</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Fresh Foods</t>
+          <t>Beverages</t>
         </is>
       </c>
       <c r="D10" t="n">
         <v>16</v>
       </c>
       <c r="E10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F10" s="1" t="n">
         <v>43831</v>
@@ -753,24 +753,24 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>{'CAT010'}</t>
+          <t>CAT010</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Bread</t>
+          <t>Water</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Bakery</t>
+          <t>Beverages</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="E11" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F11" s="1" t="n">
         <v>43831</v>
@@ -785,24 +785,24 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>{'CAT011'}</t>
+          <t>CAT011</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Cakes</t>
+          <t>Tea &amp; Coffee</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Bakery</t>
+          <t>Beverages</t>
         </is>
       </c>
       <c r="D12" t="n">
         <v>16</v>
       </c>
       <c r="E12" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F12" s="1" t="n">
         <v>43831</v>
@@ -817,17 +817,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>{'CAT012'}</t>
+          <t>CAT012</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Soft Drinks</t>
+          <t>Snacks</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Beverages</t>
+          <t>Snacks</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -849,17 +849,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>{'CAT013'}</t>
+          <t>CAT013</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Juices</t>
+          <t>Confectionery</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Beverages</t>
+          <t>Snacks</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -881,21 +881,21 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>{'CAT014'}</t>
+          <t>CAT014</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Water</t>
+          <t>Cleaning Supplies</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Beverages</t>
+          <t>Household</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="E15" t="b">
         <v>0</v>
@@ -913,17 +913,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>{'CAT015'}</t>
+          <t>CAT015</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Tea</t>
+          <t>Laundry</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Beverages</t>
+          <t>Household</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -945,17 +945,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>{'CAT016'}</t>
+          <t>CAT016</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Coffee</t>
+          <t>Kitchenware</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Beverages</t>
+          <t>Household</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -977,17 +977,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>{'CAT017'}</t>
+          <t>CAT017</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Cleaning Supplies</t>
+          <t>Personal Care</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Household</t>
+          <t>Health &amp; Beauty</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -1009,17 +1009,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>{'CAT018'}</t>
+          <t>CAT018</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Laundry</t>
+          <t>Baby Care</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Household</t>
+          <t>Health &amp; Beauty</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -1041,17 +1041,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>{'CAT019'}</t>
+          <t>CAT019</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Toiletries</t>
+          <t>Health &amp; Pharmacy</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Personal Care</t>
+          <t>Health &amp; Beauty</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -1073,17 +1073,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>{'CAT020'}</t>
+          <t>CAT020</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Baby Care</t>
+          <t>Stationery</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Personal Care</t>
+          <t>Office</t>
         </is>
       </c>
       <c r="D21" t="n">
@@ -1105,17 +1105,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>{'CAT021'}</t>
+          <t>CAT021</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Stationery</t>
+          <t>Electronics</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Office</t>
+          <t>Electronics</t>
         </is>
       </c>
       <c r="D22" t="n">
@@ -1137,17 +1137,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>{'CAT022'}</t>
+          <t>CAT022</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Electronics</t>
+          <t>Pet Care</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Electronics</t>
+          <t>Pets</t>
         </is>
       </c>
       <c r="D23" t="n">
@@ -1163,102 +1163,6 @@
         <v>46022</v>
       </c>
       <c r="H23" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>{'CAT023'}</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Kitchenware</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Home</t>
-        </is>
-      </c>
-      <c r="D24" t="n">
-        <v>16</v>
-      </c>
-      <c r="E24" t="b">
-        <v>0</v>
-      </c>
-      <c r="F24" s="1" t="n">
-        <v>43831</v>
-      </c>
-      <c r="G24" s="1" t="n">
-        <v>46022</v>
-      </c>
-      <c r="H24" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>{'CAT024'}</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Pet Food</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Pets</t>
-        </is>
-      </c>
-      <c r="D25" t="n">
-        <v>16</v>
-      </c>
-      <c r="E25" t="b">
-        <v>0</v>
-      </c>
-      <c r="F25" s="1" t="n">
-        <v>43831</v>
-      </c>
-      <c r="G25" s="1" t="n">
-        <v>46022</v>
-      </c>
-      <c r="H25" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>{'CAT025'}</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Frozen Foods</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>Frozen</t>
-        </is>
-      </c>
-      <c r="D26" t="n">
-        <v>16</v>
-      </c>
-      <c r="E26" t="b">
-        <v>1</v>
-      </c>
-      <c r="F26" s="1" t="n">
-        <v>43831</v>
-      </c>
-      <c r="G26" s="1" t="n">
-        <v>46022</v>
-      </c>
-      <c r="H26" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
created sales and sales details and they worked correctly
</commit_message>
<xml_diff>
--- a/generator/output/master/categories.xlsx
+++ b/generator/output/master/categories.xlsx
@@ -423,42 +423,42 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>category_id</t>
+          <t>CategoryID</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>category_name</t>
+          <t>CategoryName</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>category_type</t>
+          <t>CategoryType</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>tax_rate</t>
+          <t>VATRate</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>is_perishable</t>
+          <t>IsPerishable</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>created_date</t>
+          <t>CreatedDate</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>Last_updated_date</t>
+          <t>LastUpdatedDate</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>is_active</t>
+          <t>IsActive</t>
         </is>
       </c>
     </row>

</xml_diff>